<commit_message>
chỉnh sửa tên cột trong thông tin sản phẩm
</commit_message>
<xml_diff>
--- a/data/product_data/Thông tin sản phẩm.xlsx
+++ b/data/product_data/Thông tin sản phẩm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\sinvoice-creator\data\product_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E943E17-ABF5-46F1-9814-0C375C26F1D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969F18C0-8BC3-4917-ACC8-A2C4EAE74705}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD807B91-3D44-4B7C-B5DF-3904750413C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{AD807B91-3D44-4B7C-B5DF-3904750413C2}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -401,16 +401,16 @@
     <t>Mì Spaghetti 500g</t>
   </si>
   <si>
-    <t>product_code</t>
-  </si>
-  <si>
-    <t>product_name</t>
-  </si>
-  <si>
-    <t>product_unit</t>
-  </si>
-  <si>
     <t>tax_percent</t>
+  </si>
+  <si>
+    <t>item_name</t>
+  </si>
+  <si>
+    <t>item_code</t>
+  </si>
+  <si>
+    <t>item_unit</t>
   </si>
 </sst>
 </file>
@@ -805,16 +805,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B1" t="s">
         <v>123</v>
       </c>
       <c r="C1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
cập nhật thông tin sản phẩm, đổi tên cột tỉ lệ thuế
</commit_message>
<xml_diff>
--- a/data/product_data/Thông tin sản phẩm.xlsx
+++ b/data/product_data/Thông tin sản phẩm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\sinvoice-creator\data\product_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B288E78-7E17-40AA-B48B-3A8E3AED56AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4675C8-FE1A-46C7-BE5B-AB611905B6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD807B91-3D44-4B7C-B5DF-3904750413C2}"/>
   </bookViews>
@@ -353,9 +353,6 @@
     <t>Mì Spaghetti 500g</t>
   </si>
   <si>
-    <t>tax_percent</t>
-  </si>
-  <si>
     <t>item_name</t>
   </si>
   <si>
@@ -759,12 +756,18 @@
   </si>
   <si>
     <t>Túi vải O'food đỏ</t>
+  </si>
+  <si>
+    <t>tax_ratio</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -800,17 +803,17 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -1149,26 +1152,26 @@
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="88.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" t="s">
         <v>108</v>
       </c>
-      <c r="B1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -1176,13 +1179,13 @@
       <c r="C2" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>111</v>
+      <c r="A3" s="2" t="s">
+        <v>110</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -1190,13 +1193,13 @@
       <c r="C3" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>112</v>
+      <c r="A4" s="2" t="s">
+        <v>111</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
@@ -1204,13 +1207,13 @@
       <c r="C4" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>113</v>
+      <c r="A5" s="2" t="s">
+        <v>112</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -1218,13 +1221,13 @@
       <c r="C5" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>114</v>
+      <c r="A6" s="2" t="s">
+        <v>113</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
@@ -1232,13 +1235,13 @@
       <c r="C6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>115</v>
+      <c r="A7" s="2" t="s">
+        <v>114</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -1246,13 +1249,13 @@
       <c r="C7" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>116</v>
+      <c r="A8" s="2" t="s">
+        <v>115</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
@@ -1260,13 +1263,13 @@
       <c r="C8" t="s">
         <v>65</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>117</v>
+      <c r="A9" s="2" t="s">
+        <v>116</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
@@ -1274,13 +1277,13 @@
       <c r="C9" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="3">
         <v>0.05</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>118</v>
+      <c r="A10" s="2" t="s">
+        <v>117</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
@@ -1288,27 +1291,27 @@
       <c r="C10" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="3">
         <v>0.05</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>119</v>
+      <c r="A11" s="2" t="s">
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C11" t="s">
         <v>66</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>120</v>
+      <c r="A12" s="2" t="s">
+        <v>119</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
@@ -1316,27 +1319,27 @@
       <c r="C12" t="s">
         <v>65</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" t="s">
+        <v>226</v>
+      </c>
+      <c r="C13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="B13" t="s">
-        <v>227</v>
-      </c>
-      <c r="C13" t="s">
-        <v>65</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="B14" t="s">
         <v>11</v>
@@ -1344,13 +1347,13 @@
       <c r="C14" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>123</v>
+      <c r="A15" s="2" t="s">
+        <v>122</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
@@ -1358,13 +1361,13 @@
       <c r="C15" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>124</v>
+      <c r="A16" s="2" t="s">
+        <v>123</v>
       </c>
       <c r="B16" t="s">
         <v>13</v>
@@ -1372,13 +1375,13 @@
       <c r="C16" t="s">
         <v>64</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>125</v>
+      <c r="A17" s="2" t="s">
+        <v>124</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -1386,13 +1389,13 @@
       <c r="C17" t="s">
         <v>65</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>126</v>
+      <c r="A18" s="2" t="s">
+        <v>125</v>
       </c>
       <c r="B18" t="s">
         <v>15</v>
@@ -1400,13 +1403,13 @@
       <c r="C18" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>127</v>
+      <c r="A19" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="B19" t="s">
         <v>16</v>
@@ -1414,27 +1417,27 @@
       <c r="C19" t="s">
         <v>67</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B20" t="s">
+        <v>227</v>
+      </c>
+      <c r="C20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="B20" t="s">
-        <v>228</v>
-      </c>
-      <c r="C20" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="B21" t="s">
         <v>17</v>
@@ -1442,41 +1445,41 @@
       <c r="C21" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B22" t="s">
+        <v>228</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>229</v>
-      </c>
-      <c r="C22" t="s">
-        <v>65</v>
-      </c>
-      <c r="D22" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B23" t="s">
-        <v>230</v>
       </c>
       <c r="C23" t="s">
         <v>64</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>132</v>
+      <c r="A24" s="2" t="s">
+        <v>131</v>
       </c>
       <c r="B24" t="s">
         <v>18</v>
@@ -1484,13 +1487,13 @@
       <c r="C24" t="s">
         <v>65</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>133</v>
+      <c r="A25" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="B25" t="s">
         <v>19</v>
@@ -1498,13 +1501,13 @@
       <c r="C25" t="s">
         <v>65</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>134</v>
+      <c r="A26" s="2" t="s">
+        <v>133</v>
       </c>
       <c r="B26" t="s">
         <v>20</v>
@@ -1512,13 +1515,13 @@
       <c r="C26" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>135</v>
+      <c r="A27" s="2" t="s">
+        <v>134</v>
       </c>
       <c r="B27" t="s">
         <v>21</v>
@@ -1526,27 +1529,27 @@
       <c r="C27" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B28" t="s">
+        <v>230</v>
+      </c>
+      <c r="C28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="B28" t="s">
-        <v>231</v>
-      </c>
-      <c r="C28" t="s">
-        <v>65</v>
-      </c>
-      <c r="D28" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>137</v>
       </c>
       <c r="B29" t="s">
         <v>23</v>
@@ -1554,13 +1557,13 @@
       <c r="C29" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>138</v>
+      <c r="A30" s="2" t="s">
+        <v>137</v>
       </c>
       <c r="B30" t="s">
         <v>24</v>
@@ -1568,41 +1571,41 @@
       <c r="C30" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B31" t="s">
+        <v>231</v>
+      </c>
+      <c r="C31" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>232</v>
-      </c>
-      <c r="C31" t="s">
-        <v>65</v>
-      </c>
-      <c r="D31" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B32" t="s">
-        <v>233</v>
       </c>
       <c r="C32" t="s">
         <v>64</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D32" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>141</v>
+      <c r="A33" s="2" t="s">
+        <v>140</v>
       </c>
       <c r="B33" t="s">
         <v>25</v>
@@ -1610,13 +1613,13 @@
       <c r="C33" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>142</v>
+      <c r="A34" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="B34" t="s">
         <v>22</v>
@@ -1624,27 +1627,27 @@
       <c r="C34" t="s">
         <v>68</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B35" t="s">
+        <v>233</v>
+      </c>
+      <c r="C35" t="s">
+        <v>65</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="B35" t="s">
-        <v>234</v>
-      </c>
-      <c r="C35" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>144</v>
       </c>
       <c r="B36" t="s">
         <v>26</v>
@@ -1652,13 +1655,13 @@
       <c r="C36" t="s">
         <v>65</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>145</v>
+      <c r="A37" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="B37" t="s">
         <v>27</v>
@@ -1666,13 +1669,13 @@
       <c r="C37" t="s">
         <v>65</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>146</v>
+      <c r="A38" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="B38" t="s">
         <v>28</v>
@@ -1680,13 +1683,13 @@
       <c r="C38" t="s">
         <v>65</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>147</v>
+      <c r="A39" s="2" t="s">
+        <v>146</v>
       </c>
       <c r="B39" t="s">
         <v>29</v>
@@ -1694,13 +1697,13 @@
       <c r="C39" t="s">
         <v>65</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>148</v>
+      <c r="A40" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="B40" t="s">
         <v>30</v>
@@ -1708,13 +1711,13 @@
       <c r="C40" t="s">
         <v>65</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>149</v>
+      <c r="A41" s="2" t="s">
+        <v>148</v>
       </c>
       <c r="B41" t="s">
         <v>31</v>
@@ -1722,13 +1725,13 @@
       <c r="C41" t="s">
         <v>65</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>150</v>
+      <c r="A42" s="2" t="s">
+        <v>149</v>
       </c>
       <c r="B42" t="s">
         <v>32</v>
@@ -1736,13 +1739,13 @@
       <c r="C42" t="s">
         <v>68</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>151</v>
+      <c r="A43" s="2" t="s">
+        <v>150</v>
       </c>
       <c r="B43" t="s">
         <v>33</v>
@@ -1750,13 +1753,13 @@
       <c r="C43" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="1">
+      <c r="D43" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>152</v>
+      <c r="A44" s="2" t="s">
+        <v>151</v>
       </c>
       <c r="B44" t="s">
         <v>34</v>
@@ -1764,13 +1767,13 @@
       <c r="C44" t="s">
         <v>65</v>
       </c>
-      <c r="D44" s="1">
+      <c r="D44" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>153</v>
+      <c r="A45" s="2" t="s">
+        <v>152</v>
       </c>
       <c r="B45" t="s">
         <v>35</v>
@@ -1778,13 +1781,13 @@
       <c r="C45" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="1">
+      <c r="D45" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>154</v>
+      <c r="A46" s="2" t="s">
+        <v>153</v>
       </c>
       <c r="B46" t="s">
         <v>36</v>
@@ -1792,13 +1795,13 @@
       <c r="C46" t="s">
         <v>65</v>
       </c>
-      <c r="D46" s="1">
+      <c r="D46" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>155</v>
+      <c r="A47" s="2" t="s">
+        <v>154</v>
       </c>
       <c r="B47" t="s">
         <v>37</v>
@@ -1806,13 +1809,13 @@
       <c r="C47" t="s">
         <v>65</v>
       </c>
-      <c r="D47" s="1">
+      <c r="D47" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>156</v>
+      <c r="A48" s="2" t="s">
+        <v>155</v>
       </c>
       <c r="B48" t="s">
         <v>38</v>
@@ -1820,13 +1823,13 @@
       <c r="C48" t="s">
         <v>65</v>
       </c>
-      <c r="D48" s="1">
+      <c r="D48" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
-        <v>157</v>
+      <c r="A49" s="2" t="s">
+        <v>156</v>
       </c>
       <c r="B49" t="s">
         <v>39</v>
@@ -1834,13 +1837,13 @@
       <c r="C49" t="s">
         <v>65</v>
       </c>
-      <c r="D49" s="1">
+      <c r="D49" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>158</v>
+      <c r="A50" s="2" t="s">
+        <v>157</v>
       </c>
       <c r="B50" t="s">
         <v>40</v>
@@ -1848,13 +1851,13 @@
       <c r="C50" t="s">
         <v>64</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
-        <v>159</v>
+      <c r="A51" s="2" t="s">
+        <v>158</v>
       </c>
       <c r="B51" t="s">
         <v>41</v>
@@ -1862,13 +1865,13 @@
       <c r="C51" t="s">
         <v>68</v>
       </c>
-      <c r="D51" s="1">
+      <c r="D51" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
-        <v>160</v>
+      <c r="A52" s="2" t="s">
+        <v>159</v>
       </c>
       <c r="B52" t="s">
         <v>42</v>
@@ -1876,13 +1879,13 @@
       <c r="C52" t="s">
         <v>65</v>
       </c>
-      <c r="D52" s="1">
+      <c r="D52" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
-        <v>161</v>
+      <c r="A53" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="B53" t="s">
         <v>43</v>
@@ -1890,13 +1893,13 @@
       <c r="C53" t="s">
         <v>65</v>
       </c>
-      <c r="D53" s="1">
+      <c r="D53" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
-        <v>162</v>
+      <c r="A54" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="B54" t="s">
         <v>44</v>
@@ -1904,13 +1907,13 @@
       <c r="C54" t="s">
         <v>68</v>
       </c>
-      <c r="D54" s="1">
+      <c r="D54" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
-        <v>163</v>
+      <c r="A55" s="2" t="s">
+        <v>162</v>
       </c>
       <c r="B55" t="s">
         <v>45</v>
@@ -1918,13 +1921,13 @@
       <c r="C55" t="s">
         <v>68</v>
       </c>
-      <c r="D55" s="1">
+      <c r="D55" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="3" t="s">
-        <v>164</v>
+      <c r="A56" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="B56" t="s">
         <v>46</v>
@@ -1932,13 +1935,13 @@
       <c r="C56" t="s">
         <v>65</v>
       </c>
-      <c r="D56" s="1">
+      <c r="D56" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
-        <v>165</v>
+      <c r="A57" s="2" t="s">
+        <v>164</v>
       </c>
       <c r="B57" t="s">
         <v>47</v>
@@ -1946,13 +1949,13 @@
       <c r="C57" t="s">
         <v>65</v>
       </c>
-      <c r="D57" s="1">
+      <c r="D57" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="3" t="s">
-        <v>166</v>
+      <c r="A58" s="2" t="s">
+        <v>165</v>
       </c>
       <c r="B58" t="s">
         <v>49</v>
@@ -1960,13 +1963,13 @@
       <c r="C58" t="s">
         <v>65</v>
       </c>
-      <c r="D58" s="1">
+      <c r="D58" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="3" t="s">
-        <v>167</v>
+      <c r="A59" s="2" t="s">
+        <v>166</v>
       </c>
       <c r="B59" t="s">
         <v>48</v>
@@ -1974,13 +1977,13 @@
       <c r="C59" t="s">
         <v>65</v>
       </c>
-      <c r="D59" s="1">
+      <c r="D59" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>168</v>
+      <c r="A60" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="B60" t="s">
         <v>50</v>
@@ -1988,13 +1991,13 @@
       <c r="C60" t="s">
         <v>65</v>
       </c>
-      <c r="D60" s="1">
+      <c r="D60" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
-        <v>169</v>
+      <c r="A61" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="B61" t="s">
         <v>51</v>
@@ -2002,27 +2005,27 @@
       <c r="C61" t="s">
         <v>65</v>
       </c>
-      <c r="D61" s="1">
+      <c r="D61" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="3" t="s">
+      <c r="A62" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B62" t="s">
+        <v>234</v>
+      </c>
+      <c r="C62" t="s">
+        <v>65</v>
+      </c>
+      <c r="D62" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="B62" t="s">
-        <v>235</v>
-      </c>
-      <c r="C62" t="s">
-        <v>65</v>
-      </c>
-      <c r="D62" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="3" t="s">
-        <v>171</v>
       </c>
       <c r="B63" t="s">
         <v>52</v>
@@ -2030,13 +2033,13 @@
       <c r="C63" t="s">
         <v>65</v>
       </c>
-      <c r="D63" s="1">
+      <c r="D63" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
-        <v>172</v>
+      <c r="A64" s="2" t="s">
+        <v>171</v>
       </c>
       <c r="B64" t="s">
         <v>53</v>
@@ -2044,27 +2047,27 @@
       <c r="C64" t="s">
         <v>65</v>
       </c>
-      <c r="D64" s="1">
+      <c r="D64" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B65" t="s">
+        <v>235</v>
+      </c>
+      <c r="C65" t="s">
+        <v>65</v>
+      </c>
+      <c r="D65" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="B65" t="s">
-        <v>236</v>
-      </c>
-      <c r="C65" t="s">
-        <v>65</v>
-      </c>
-      <c r="D65" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="3" t="s">
-        <v>174</v>
       </c>
       <c r="B66" t="s">
         <v>54</v>
@@ -2072,13 +2075,13 @@
       <c r="C66" t="s">
         <v>65</v>
       </c>
-      <c r="D66" s="1">
+      <c r="D66" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="3" t="s">
-        <v>175</v>
+      <c r="A67" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="B67" t="s">
         <v>55</v>
@@ -2086,13 +2089,13 @@
       <c r="C67" t="s">
         <v>65</v>
       </c>
-      <c r="D67" s="1">
+      <c r="D67" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="3" t="s">
-        <v>176</v>
+      <c r="A68" s="2" t="s">
+        <v>175</v>
       </c>
       <c r="B68" t="s">
         <v>56</v>
@@ -2100,13 +2103,13 @@
       <c r="C68" t="s">
         <v>65</v>
       </c>
-      <c r="D68" s="1">
+      <c r="D68" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="3" t="s">
-        <v>177</v>
+      <c r="A69" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="B69" t="s">
         <v>0</v>
@@ -2114,13 +2117,13 @@
       <c r="C69" t="s">
         <v>65</v>
       </c>
-      <c r="D69" s="1">
+      <c r="D69" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="3" t="s">
-        <v>178</v>
+      <c r="A70" s="2" t="s">
+        <v>177</v>
       </c>
       <c r="B70" t="s">
         <v>57</v>
@@ -2128,13 +2131,13 @@
       <c r="C70" t="s">
         <v>66</v>
       </c>
-      <c r="D70" s="1">
+      <c r="D70" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="3" t="s">
-        <v>179</v>
+      <c r="A71" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="B71" t="s">
         <v>58</v>
@@ -2142,13 +2145,13 @@
       <c r="C71" t="s">
         <v>66</v>
       </c>
-      <c r="D71" s="1">
+      <c r="D71" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="3" t="s">
-        <v>180</v>
+      <c r="A72" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="B72" t="s">
         <v>59</v>
@@ -2156,13 +2159,13 @@
       <c r="C72" t="s">
         <v>69</v>
       </c>
-      <c r="D72" s="1">
+      <c r="D72" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="3" t="s">
-        <v>181</v>
+      <c r="A73" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="B73" t="s">
         <v>60</v>
@@ -2170,27 +2173,27 @@
       <c r="C73" t="s">
         <v>65</v>
       </c>
-      <c r="D73" s="1">
+      <c r="D73" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="3" t="s">
-        <v>182</v>
+      <c r="A74" s="2" t="s">
+        <v>181</v>
       </c>
       <c r="B74" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C74" t="s">
         <v>64</v>
       </c>
-      <c r="D74" s="1">
+      <c r="D74" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="3" t="s">
-        <v>183</v>
+      <c r="A75" s="2" t="s">
+        <v>182</v>
       </c>
       <c r="B75" t="s">
         <v>61</v>
@@ -2198,13 +2201,13 @@
       <c r="C75" t="s">
         <v>69</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D75" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="3" t="s">
-        <v>184</v>
+      <c r="A76" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="B76" t="s">
         <v>62</v>
@@ -2212,13 +2215,13 @@
       <c r="C76" t="s">
         <v>65</v>
       </c>
-      <c r="D76" s="1">
+      <c r="D76" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="3" t="s">
-        <v>185</v>
+      <c r="A77" s="2" t="s">
+        <v>184</v>
       </c>
       <c r="B77" t="s">
         <v>63</v>
@@ -2226,27 +2229,27 @@
       <c r="C77" t="s">
         <v>65</v>
       </c>
-      <c r="D77" s="1">
+      <c r="D77" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="3" t="s">
-        <v>186</v>
+      <c r="A78" s="2" t="s">
+        <v>185</v>
       </c>
       <c r="B78" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C78" t="s">
         <v>64</v>
       </c>
-      <c r="D78" s="1">
+      <c r="D78" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="3" t="s">
-        <v>187</v>
+      <c r="A79" s="2" t="s">
+        <v>186</v>
       </c>
       <c r="B79" t="s">
         <v>70</v>
@@ -2254,13 +2257,13 @@
       <c r="C79" t="s">
         <v>65</v>
       </c>
-      <c r="D79" s="1">
+      <c r="D79" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="3" t="s">
-        <v>188</v>
+      <c r="A80" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="B80" t="s">
         <v>71</v>
@@ -2268,13 +2271,13 @@
       <c r="C80" t="s">
         <v>65</v>
       </c>
-      <c r="D80" s="1">
+      <c r="D80" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="3" t="s">
-        <v>189</v>
+      <c r="A81" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="B81" t="s">
         <v>72</v>
@@ -2282,13 +2285,13 @@
       <c r="C81" t="s">
         <v>68</v>
       </c>
-      <c r="D81" s="1">
+      <c r="D81" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="3" t="s">
-        <v>190</v>
+      <c r="A82" s="2" t="s">
+        <v>189</v>
       </c>
       <c r="B82" t="s">
         <v>73</v>
@@ -2296,13 +2299,13 @@
       <c r="C82" t="s">
         <v>68</v>
       </c>
-      <c r="D82" s="1">
+      <c r="D82" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="3" t="s">
-        <v>191</v>
+      <c r="A83" s="2" t="s">
+        <v>190</v>
       </c>
       <c r="B83" t="s">
         <v>74</v>
@@ -2310,13 +2313,13 @@
       <c r="C83" t="s">
         <v>69</v>
       </c>
-      <c r="D83" s="1">
+      <c r="D83" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="3" t="s">
-        <v>192</v>
+      <c r="A84" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="B84" t="s">
         <v>75</v>
@@ -2324,13 +2327,13 @@
       <c r="C84" t="s">
         <v>65</v>
       </c>
-      <c r="D84" s="1">
+      <c r="D84" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="3" t="s">
-        <v>193</v>
+      <c r="A85" s="2" t="s">
+        <v>192</v>
       </c>
       <c r="B85" t="s">
         <v>76</v>
@@ -2338,13 +2341,13 @@
       <c r="C85" t="s">
         <v>65</v>
       </c>
-      <c r="D85" s="1">
+      <c r="D85" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="3" t="s">
-        <v>194</v>
+      <c r="A86" s="2" t="s">
+        <v>193</v>
       </c>
       <c r="B86" t="s">
         <v>77</v>
@@ -2352,13 +2355,13 @@
       <c r="C86" t="s">
         <v>65</v>
       </c>
-      <c r="D86" s="1">
+      <c r="D86" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="3" t="s">
-        <v>195</v>
+      <c r="A87" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="B87" t="s">
         <v>78</v>
@@ -2366,13 +2369,13 @@
       <c r="C87" t="s">
         <v>64</v>
       </c>
-      <c r="D87" s="1">
+      <c r="D87" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="3" t="s">
-        <v>196</v>
+      <c r="A88" s="2" t="s">
+        <v>195</v>
       </c>
       <c r="B88" t="s">
         <v>79</v>
@@ -2380,13 +2383,13 @@
       <c r="C88" t="s">
         <v>65</v>
       </c>
-      <c r="D88" s="1">
+      <c r="D88" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="3" t="s">
-        <v>197</v>
+      <c r="A89" s="2" t="s">
+        <v>196</v>
       </c>
       <c r="B89" t="s">
         <v>80</v>
@@ -2394,13 +2397,13 @@
       <c r="C89" t="s">
         <v>64</v>
       </c>
-      <c r="D89" s="1">
+      <c r="D89" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="3" t="s">
-        <v>198</v>
+      <c r="A90" s="2" t="s">
+        <v>197</v>
       </c>
       <c r="B90" t="s">
         <v>81</v>
@@ -2408,13 +2411,13 @@
       <c r="C90" t="s">
         <v>64</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D90" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="3" t="s">
-        <v>199</v>
+      <c r="A91" s="2" t="s">
+        <v>198</v>
       </c>
       <c r="B91" t="s">
         <v>82</v>
@@ -2422,13 +2425,13 @@
       <c r="C91" t="s">
         <v>68</v>
       </c>
-      <c r="D91" s="1">
+      <c r="D91" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="3" t="s">
-        <v>200</v>
+      <c r="A92" s="2" t="s">
+        <v>199</v>
       </c>
       <c r="B92" t="s">
         <v>83</v>
@@ -2436,13 +2439,13 @@
       <c r="C92" t="s">
         <v>64</v>
       </c>
-      <c r="D92" s="1">
+      <c r="D92" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="3" t="s">
-        <v>201</v>
+      <c r="A93" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="B93" t="s">
         <v>84</v>
@@ -2450,13 +2453,13 @@
       <c r="C93" t="s">
         <v>65</v>
       </c>
-      <c r="D93" s="1">
+      <c r="D93" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="3" t="s">
-        <v>202</v>
+      <c r="A94" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="B94" t="s">
         <v>85</v>
@@ -2464,13 +2467,13 @@
       <c r="C94" t="s">
         <v>65</v>
       </c>
-      <c r="D94" s="1">
+      <c r="D94" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="3" t="s">
-        <v>203</v>
+      <c r="A95" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="B95" t="s">
         <v>86</v>
@@ -2478,13 +2481,13 @@
       <c r="C95" t="s">
         <v>65</v>
       </c>
-      <c r="D95" s="1">
+      <c r="D95" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="3" t="s">
-        <v>204</v>
+      <c r="A96" s="2" t="s">
+        <v>203</v>
       </c>
       <c r="B96" t="s">
         <v>87</v>
@@ -2492,13 +2495,13 @@
       <c r="C96" t="s">
         <v>64</v>
       </c>
-      <c r="D96" s="1">
+      <c r="D96" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="3" t="s">
-        <v>205</v>
+      <c r="A97" s="2" t="s">
+        <v>204</v>
       </c>
       <c r="B97" t="s">
         <v>88</v>
@@ -2506,13 +2509,13 @@
       <c r="C97" t="s">
         <v>65</v>
       </c>
-      <c r="D97" s="1">
+      <c r="D97" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="3" t="s">
-        <v>206</v>
+      <c r="A98" s="2" t="s">
+        <v>205</v>
       </c>
       <c r="B98" t="s">
         <v>89</v>
@@ -2520,13 +2523,13 @@
       <c r="C98" t="s">
         <v>65</v>
       </c>
-      <c r="D98" s="1">
+      <c r="D98" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="3" t="s">
-        <v>207</v>
+      <c r="A99" s="2" t="s">
+        <v>206</v>
       </c>
       <c r="B99" t="s">
         <v>90</v>
@@ -2534,13 +2537,13 @@
       <c r="C99" t="s">
         <v>64</v>
       </c>
-      <c r="D99" s="1">
+      <c r="D99" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="3" t="s">
-        <v>208</v>
+      <c r="A100" s="2" t="s">
+        <v>207</v>
       </c>
       <c r="B100" t="s">
         <v>91</v>
@@ -2548,13 +2551,13 @@
       <c r="C100" t="s">
         <v>64</v>
       </c>
-      <c r="D100" s="1">
+      <c r="D100" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="3" t="s">
-        <v>209</v>
+      <c r="A101" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="B101" t="s">
         <v>92</v>
@@ -2562,13 +2565,13 @@
       <c r="C101" t="s">
         <v>64</v>
       </c>
-      <c r="D101" s="1">
+      <c r="D101" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="3" t="s">
-        <v>210</v>
+      <c r="A102" s="2" t="s">
+        <v>209</v>
       </c>
       <c r="B102" t="s">
         <v>93</v>
@@ -2576,13 +2579,13 @@
       <c r="C102" t="s">
         <v>65</v>
       </c>
-      <c r="D102" s="1">
+      <c r="D102" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="3" t="s">
-        <v>211</v>
+      <c r="A103" s="2" t="s">
+        <v>210</v>
       </c>
       <c r="B103" t="s">
         <v>94</v>
@@ -2590,13 +2593,13 @@
       <c r="C103" t="s">
         <v>65</v>
       </c>
-      <c r="D103" s="1">
+      <c r="D103" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="3" t="s">
-        <v>212</v>
+      <c r="A104" s="2" t="s">
+        <v>211</v>
       </c>
       <c r="B104" t="s">
         <v>95</v>
@@ -2604,13 +2607,13 @@
       <c r="C104" t="s">
         <v>64</v>
       </c>
-      <c r="D104" s="1">
+      <c r="D104" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="3" t="s">
-        <v>213</v>
+      <c r="A105" s="2" t="s">
+        <v>212</v>
       </c>
       <c r="B105" t="s">
         <v>96</v>
@@ -2618,13 +2621,13 @@
       <c r="C105" t="s">
         <v>64</v>
       </c>
-      <c r="D105" s="1">
+      <c r="D105" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="3" t="s">
-        <v>214</v>
+      <c r="A106" s="2" t="s">
+        <v>213</v>
       </c>
       <c r="B106" t="s">
         <v>97</v>
@@ -2632,13 +2635,13 @@
       <c r="C106" t="s">
         <v>64</v>
       </c>
-      <c r="D106" s="1">
+      <c r="D106" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
-        <v>215</v>
+      <c r="A107" s="2" t="s">
+        <v>214</v>
       </c>
       <c r="B107" t="s">
         <v>98</v>
@@ -2646,13 +2649,13 @@
       <c r="C107" t="s">
         <v>65</v>
       </c>
-      <c r="D107" s="1">
+      <c r="D107" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="3" t="s">
-        <v>216</v>
+      <c r="A108" s="2" t="s">
+        <v>215</v>
       </c>
       <c r="B108" t="s">
         <v>99</v>
@@ -2660,13 +2663,13 @@
       <c r="C108" t="s">
         <v>65</v>
       </c>
-      <c r="D108" s="1">
+      <c r="D108" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="3" t="s">
-        <v>217</v>
+      <c r="A109" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="B109" t="s">
         <v>100</v>
@@ -2674,13 +2677,13 @@
       <c r="C109" t="s">
         <v>65</v>
       </c>
-      <c r="D109" s="1">
+      <c r="D109" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A110" s="3" t="s">
-        <v>218</v>
+      <c r="A110" s="2" t="s">
+        <v>217</v>
       </c>
       <c r="B110" t="s">
         <v>101</v>
@@ -2688,13 +2691,13 @@
       <c r="C110" t="s">
         <v>65</v>
       </c>
-      <c r="D110" s="1">
+      <c r="D110" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A111" s="3" t="s">
-        <v>219</v>
+      <c r="A111" s="2" t="s">
+        <v>218</v>
       </c>
       <c r="B111" t="s">
         <v>102</v>
@@ -2702,13 +2705,13 @@
       <c r="C111" t="s">
         <v>65</v>
       </c>
-      <c r="D111" s="1">
+      <c r="D111" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" s="3" t="s">
-        <v>220</v>
+      <c r="A112" s="2" t="s">
+        <v>219</v>
       </c>
       <c r="B112" t="s">
         <v>103</v>
@@ -2716,13 +2719,13 @@
       <c r="C112" t="s">
         <v>65</v>
       </c>
-      <c r="D112" s="1">
+      <c r="D112" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A113" s="3" t="s">
-        <v>221</v>
+      <c r="A113" s="2" t="s">
+        <v>220</v>
       </c>
       <c r="B113" t="s">
         <v>104</v>
@@ -2730,55 +2733,55 @@
       <c r="C113" t="s">
         <v>64</v>
       </c>
-      <c r="D113" s="1">
+      <c r="D113" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A114" s="3" t="s">
+      <c r="A114" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B114" t="s">
+        <v>238</v>
+      </c>
+      <c r="C114" t="s">
+        <v>65</v>
+      </c>
+      <c r="D114" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B115" t="s">
         <v>239</v>
       </c>
-      <c r="C114" t="s">
-        <v>65</v>
-      </c>
-      <c r="D114" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="3" t="s">
+      <c r="C115" t="s">
+        <v>65</v>
+      </c>
+      <c r="D115" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B116" t="s">
         <v>240</v>
-      </c>
-      <c r="C115" t="s">
-        <v>65</v>
-      </c>
-      <c r="D115" s="1">
-        <v>0.08</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A116" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="B116" t="s">
-        <v>241</v>
       </c>
       <c r="C116" t="s">
         <v>66</v>
       </c>
-      <c r="D116" s="1">
+      <c r="D116" s="3">
         <v>0.08</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A117" s="3" t="s">
-        <v>225</v>
+      <c r="A117" s="2" t="s">
+        <v>224</v>
       </c>
       <c r="B117" t="s">
         <v>105</v>
@@ -2786,10 +2789,10 @@
       <c r="C117" t="s">
         <v>65</v>
       </c>
-      <c r="D117" s="2">
-        <v>0.08</v>
-      </c>
-      <c r="E117" s="2"/>
+      <c r="D117" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="E117" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576 G1:G1048576">

</xml_diff>

<commit_message>
sửa lỗi logic kiểm tra sản phẩm thiếu
</commit_message>
<xml_diff>
--- a/data/product_data/Thông tin sản phẩm.xlsx
+++ b/data/product_data/Thông tin sản phẩm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\sinvoice-creator\data\product_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\sinvoice-creator\data\product_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A4675C8-FE1A-46C7-BE5B-AB611905B6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A523E5E4-5794-4EB6-9843-33394610BA8F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD807B91-3D44-4B7C-B5DF-3904750413C2}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="243">
   <si>
     <t>Lá Kim cuốn cơm 10g*64EA (HD)</t>
   </si>
@@ -759,6 +759,9 @@
   </si>
   <si>
     <t>tax_ratio</t>
+  </si>
+  <si>
+    <t>Cốc O’food mừng đại lễ + Ecom</t>
   </si>
 </sst>
 </file>
@@ -850,9 +853,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -890,7 +893,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -996,7 +999,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1138,7 +1141,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1146,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EAB637-782F-4865-843F-5C89801F0A39}">
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -2794,6 +2797,20 @@
       </c>
       <c r="E117" s="1"/>
     </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118">
+        <v>2152508</v>
+      </c>
+      <c r="B118" t="s">
+        <v>242</v>
+      </c>
+      <c r="C118" t="s">
+        <v>67</v>
+      </c>
+      <c r="D118" s="3">
+        <v>0.08</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:A1048576 G1:G1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="3"/>

</xml_diff>